<commit_message>
[UI] TitleUI 레이아웃 구성
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/CBAEnding.xlsx
+++ b/JsonConverter/ExcelFiles/CBAEnding.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameProjects\CBA\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388F0C03-8167-4DA8-8CAE-1DF4940AF2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB225A74-89EE-425C-A335-5CB51A908105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15480" yWindow="1610" windowWidth="14740" windowHeight="12440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1650" yWindow="2205" windowWidth="24660" windowHeight="12435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CBAEndingData" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>string</t>
   </si>
@@ -73,6 +73,18 @@
   </si>
   <si>
     <t>엉뚱곰은 집으로 돌아갔다.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>엔딩제목</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>엔딩설명</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>성공여부</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -550,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -560,58 +572,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="27">
-      <c r="A3" s="9" t="s">
+    <row r="4" spans="1:4" ht="27">
+      <c r="A4" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="9" t="b">
+      <c r="D4" s="9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="12" t="s">
+    <row r="5" spans="1:4">
+      <c r="A5" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="12" t="b">
+      <c r="D5" s="12" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[Asset] 스페셜 이벤트 배경 BG_Meadow, BG_Forest 추가
+기타 데이터 정리
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/CBAEnding.xlsx
+++ b/JsonConverter/ExcelFiles/CBAEnding.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameProjects\CBA\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD95CDF-4AC6-4878-A937-91DFB1DB7200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5B49AC-E96F-4906-BE8B-147544BD57FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -144,11 +144,11 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>곰순씨의 마음을 얻었지만..</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>곰순씨에게도 차였고…</t>
+    <t xml:space="preserve"> 곰순씨의 마음을 얻었지만..</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> 곰순씨에게도 차였고…</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -634,10 +634,10 @@
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="45" style="1" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="14.125" customWidth="1"/>
+    <col min="5" max="5" width="20.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">

</xml_diff>